<commit_message>
Batch 1: 10 PFE application drafts; flag emails to verify
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014L6ZvGt8TCo7GsJyTNk89Z
</commit_message>
<xml_diff>
--- a/Copie de stage.xlsx
+++ b/Copie de stage.xlsx
@@ -699,27 +699,27 @@
         <v>45957.43643427084</v>
       </c>
       <c r="M2" s="29" t="n"/>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P2" s="0" t="inlineStr">
         <is>
           <t>anglais</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q2" s="0" t="inlineStr">
         <is>
           <t>STM32N6 (IA embarquée) ; CAN Bus ; SunWhirl</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R2" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:05</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S2" s="0" t="inlineStr">
         <is>
           <t>CV_EN.pdf</t>
         </is>
@@ -765,6 +765,31 @@
         <v>45957.43644045139</v>
       </c>
       <c r="M3" s="29" t="n"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>STM32N6 (IA embarquée) ; CAN Bus ; CalmaWear</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:32</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="22.5" customHeight="1" s="32">
       <c r="A4" s="31" t="inlineStr">
@@ -810,6 +835,31 @@
         <v>45957.43644534722</v>
       </c>
       <c r="M4" s="29" t="n"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>MIGSens ; CAN Bus ; Télésurveillance temps réel</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:32</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22.5" customHeight="1" s="32">
       <c r="A5" s="31" t="inlineStr">
@@ -874,6 +924,31 @@
         <v>45957.43645006944</v>
       </c>
       <c r="M6" s="29" t="n"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>MPPT (Simulink) ; Micro-réseaux PES/PELS ; SunWhirl</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:32</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="22.5" customHeight="1" s="32">
       <c r="A7" s="31" t="inlineStr">
@@ -942,27 +1017,27 @@
         <v>45957.43650123842</v>
       </c>
       <c r="M8" s="29" t="n"/>
-      <c r="O8" t="inlineStr">
+      <c r="O8" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="P8" s="0" t="inlineStr">
         <is>
           <t>anglais</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="Q8" s="0" t="inlineStr">
         <is>
           <t>Télésurveillance temps réel ; CAN Bus ; SunWhirl</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="R8" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:05</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="S8" s="0" t="inlineStr">
         <is>
           <t>CV_EN.pdf</t>
         </is>
@@ -1039,6 +1114,31 @@
         <v>45957.4365062963</v>
       </c>
       <c r="M10" s="29" t="n"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Télésurveillance temps réel ; CAN Bus ; CalmaWear</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:32</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="22.5" customHeight="1" s="32">
       <c r="A11" s="31" t="inlineStr">
@@ -1084,6 +1184,11 @@
         <v>45957.43651159723</v>
       </c>
       <c r="M11" s="29" t="n"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="22.5" customHeight="1" s="32">
       <c r="A12" s="31" t="inlineStr">
@@ -1123,6 +1228,31 @@
         <v>45957.43651789352</v>
       </c>
       <c r="M12" s="29" t="n"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>anglais</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>CAN Bus ; Sagemcom ; SunWhirl (+ H2GP)</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:32</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>CV_EN.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="22.5" customHeight="1" s="32">
       <c r="A13" s="31" t="inlineStr">
@@ -1168,6 +1298,11 @@
         <v>45957.43654626158</v>
       </c>
       <c r="M13" s="29" t="n"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="22.5" customHeight="1" s="32">
       <c r="A14" s="31" t="inlineStr">
@@ -1211,6 +1346,11 @@
         <v>45957.43655104167</v>
       </c>
       <c r="M14" s="29" t="n"/>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="22.5" customHeight="1" s="32">
       <c r="A15" s="31" t="inlineStr">
@@ -1256,6 +1396,31 @@
         <v>45957.43655642361</v>
       </c>
       <c r="M15" s="29" t="n"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Micro-réseaux PES/PELS ; MPPT ; SunWhirl</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:32</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="22.5" customHeight="1" s="32">
       <c r="A16" s="31" t="inlineStr">
@@ -1289,6 +1454,11 @@
         <v>45957.4365615162</v>
       </c>
       <c r="M16" s="29" t="n"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="22.5" customHeight="1" s="32">
       <c r="A17" s="31" t="inlineStr">
@@ -1330,6 +1500,31 @@
         <v>45957.4366125926</v>
       </c>
       <c r="M17" s="29" t="n"/>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Sagemcom ; MPPT ; MIGSens</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:32</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="22.5" customHeight="1" s="32">
       <c r="A18" s="31" t="inlineStr">
@@ -1371,6 +1566,31 @@
         <v>45957.43661765046</v>
       </c>
       <c r="M18" s="29" t="n"/>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Micro-réseaux PES/PELS ; MIGSens ; SunWhirl (+ H2GP)</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:32</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="22.5" customHeight="1" s="32">
       <c r="A19" s="31" t="inlineStr">
@@ -1408,6 +1628,11 @@
         <v>45957.43662319444</v>
       </c>
       <c r="M19" s="29" t="n"/>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="22.5" customHeight="1" s="32">
       <c r="A20" s="31" t="inlineStr">
@@ -1449,6 +1674,11 @@
         <v>45957.43662777778</v>
       </c>
       <c r="M20" s="29" t="n"/>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="22.5" customHeight="1" s="32">
       <c r="A21" s="31" t="inlineStr">
@@ -1513,6 +1743,11 @@
         <v>45957.43667891204</v>
       </c>
       <c r="M22" s="29" t="n"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="22.5" customHeight="1" s="32">
       <c r="A23" s="31" t="inlineStr">
@@ -1669,6 +1904,11 @@
         <v>45957.43668399306</v>
       </c>
       <c r="M28" s="29" t="n"/>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="22.5" customHeight="1" s="32">
       <c r="A29" s="31" t="inlineStr">
@@ -1706,6 +1946,31 @@
         <v>45957.43668935185</v>
       </c>
       <c r="M29" s="29" t="n"/>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>anglais</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>SunWhirl ; CAN Bus ; STM32N6 (IA embarquée)</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:32</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>CV_EN.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="22.5" customHeight="1" s="32">
       <c r="A30" s="31" t="inlineStr">
@@ -1739,6 +2004,11 @@
         <v>45957.43669423611</v>
       </c>
       <c r="M30" s="29" t="n"/>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="22.5" customHeight="1" s="32">
       <c r="A31" s="31" t="inlineStr">
@@ -1845,6 +2115,11 @@
         <v>45957.43672258102</v>
       </c>
       <c r="M34" s="29" t="n"/>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="22.5" customHeight="1" s="32">
       <c r="A35" s="31" t="inlineStr">
@@ -1882,6 +2157,11 @@
         <v>45957.43672762731</v>
       </c>
       <c r="M35" s="29" t="n"/>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="22.5" customHeight="1" s="32">
       <c r="A36" s="31" t="inlineStr">
@@ -1920,6 +2200,31 @@
         <v>45957.4367333449</v>
       </c>
       <c r="M36" s="29" t="n"/>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>anglais</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>CAN Bus ; MIGSens ; CalmaWear</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:32</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>CV_EN.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="22.5" customHeight="1" s="32">
       <c r="A37" s="31" t="inlineStr">
@@ -1965,6 +2270,11 @@
         <v>45957.43673850694</v>
       </c>
       <c r="M37" s="29" t="n"/>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="22.5" customHeight="1" s="32">
       <c r="A38" s="31" t="inlineStr">
@@ -2085,6 +2395,11 @@
         <v>45957.43679489583</v>
       </c>
       <c r="M41" s="29" t="n"/>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="22.5" customHeight="1" s="32">
       <c r="A42" s="31" t="inlineStr">
@@ -2118,6 +2433,11 @@
         <v>45957.43679978009</v>
       </c>
       <c r="M42" s="29" t="n"/>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="22.5" customHeight="1" s="32">
       <c r="A43" s="31" t="inlineStr">
@@ -2178,6 +2498,11 @@
         <v>45957.43680464121</v>
       </c>
       <c r="M44" s="29" t="n"/>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="22.5" customHeight="1" s="32">
       <c r="A45" s="31" t="inlineStr">
@@ -2211,6 +2536,11 @@
         <v>45957.4369069676</v>
       </c>
       <c r="M45" s="29" t="n"/>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="22.5" customHeight="1" s="32">
       <c r="A46" s="31" t="inlineStr">
@@ -2464,6 +2794,11 @@
         <v>45957.43706625</v>
       </c>
       <c r="M53" s="29" t="n"/>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="22.5" customHeight="1" s="32">
       <c r="A54" s="31" t="inlineStr">
@@ -2497,6 +2832,11 @@
         <v>45957.43711337963</v>
       </c>
       <c r="M54" s="29" t="n"/>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="22.5" customHeight="1" s="32">
       <c r="A55" s="31" t="inlineStr">
@@ -2676,6 +3016,11 @@
         <v>45957.43719201389</v>
       </c>
       <c r="M59" s="29" t="n"/>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="22.5" customHeight="1" s="32">
       <c r="A60" s="31" t="inlineStr">
@@ -2811,27 +3156,27 @@
         <v>45957.43730099537</v>
       </c>
       <c r="M62" s="29" t="n"/>
-      <c r="O62" t="inlineStr">
+      <c r="O62" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P62" t="inlineStr">
+      <c r="P62" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q62" t="inlineStr">
+      <c r="Q62" s="0" t="inlineStr">
         <is>
           <t>Sagemcom (onduleur PV) ; SunWhirl ; MIGSens</t>
         </is>
       </c>
-      <c r="R62" t="inlineStr">
+      <c r="R62" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:05</t>
         </is>
       </c>
-      <c r="S62" t="inlineStr">
+      <c r="S62" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -3067,6 +3412,11 @@
         <v>45957.43740361111</v>
       </c>
       <c r="M69" s="29" t="n"/>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="22.5" customHeight="1" s="32">
       <c r="A70" s="31" t="inlineStr">
@@ -3210,6 +3560,11 @@
         <v>45988.51455915509</v>
       </c>
       <c r="M74" s="29" t="n"/>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="22.5" customHeight="1" s="32">
       <c r="A75" s="31" t="inlineStr">
@@ -3243,6 +3598,11 @@
         <v>45988.51456922454</v>
       </c>
       <c r="M75" s="29" t="n"/>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="22.5" customHeight="1" s="32">
       <c r="A76" s="31" t="inlineStr">
@@ -3416,6 +3776,11 @@
       <c r="L81" s="30" t="n">
         <v>45988.51463702547</v>
       </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="22.5" customHeight="1" s="32">
       <c r="A82" s="31" t="inlineStr">
@@ -3476,6 +3841,11 @@
       <c r="L83" s="30" t="n">
         <v>45988.51468505787</v>
       </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="22.5" customHeight="1" s="32">
       <c r="A84" s="19" t="inlineStr">
@@ -3506,6 +3876,11 @@
       <c r="L84" s="30" t="n">
         <v>45988.51470270834</v>
       </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="22.5" customHeight="1" s="32">
       <c r="A85" s="31" t="inlineStr">
@@ -3536,6 +3911,11 @@
       <c r="L85" s="30" t="n">
         <v>45988.51471092593</v>
       </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="22.5" customHeight="1" s="32">
       <c r="A86" s="31" t="inlineStr">
@@ -3625,6 +4005,11 @@
       </c>
       <c r="L88" s="30" t="n">
         <v>45995.67262321759</v>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>email à vérifier</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Batch 2: 10 PFE application drafts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014L6ZvGt8TCo7GsJyTNk89Z
</commit_message>
<xml_diff>
--- a/Copie de stage.xlsx
+++ b/Copie de stage.xlsx
@@ -765,27 +765,27 @@
         <v>45957.43644045139</v>
       </c>
       <c r="M3" s="29" t="n"/>
-      <c r="O3" t="inlineStr">
+      <c r="O3" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P3" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q3" s="0" t="inlineStr">
         <is>
           <t>STM32N6 (IA embarquée) ; CAN Bus ; CalmaWear</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R3" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:32</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S3" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -835,27 +835,27 @@
         <v>45957.43644534722</v>
       </c>
       <c r="M4" s="29" t="n"/>
-      <c r="O4" t="inlineStr">
+      <c r="O4" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P4" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q4" s="0" t="inlineStr">
         <is>
           <t>MIGSens ; CAN Bus ; Télésurveillance temps réel</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R4" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:32</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S4" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -924,27 +924,27 @@
         <v>45957.43645006944</v>
       </c>
       <c r="M6" s="29" t="n"/>
-      <c r="O6" t="inlineStr">
+      <c r="O6" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="P6" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="Q6" s="0" t="inlineStr">
         <is>
           <t>MPPT (Simulink) ; Micro-réseaux PES/PELS ; SunWhirl</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="R6" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:32</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="S6" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -1114,27 +1114,27 @@
         <v>45957.4365062963</v>
       </c>
       <c r="M10" s="29" t="n"/>
-      <c r="O10" t="inlineStr">
+      <c r="O10" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="P10" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="Q10" s="0" t="inlineStr">
         <is>
           <t>Télésurveillance temps réel ; CAN Bus ; CalmaWear</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="R10" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:32</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="S10" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -1184,7 +1184,7 @@
         <v>45957.43651159723</v>
       </c>
       <c r="M11" s="29" t="n"/>
-      <c r="O11" t="inlineStr">
+      <c r="O11" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -1228,27 +1228,27 @@
         <v>45957.43651789352</v>
       </c>
       <c r="M12" s="29" t="n"/>
-      <c r="O12" t="inlineStr">
+      <c r="O12" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="P12" s="0" t="inlineStr">
         <is>
           <t>anglais</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="Q12" s="0" t="inlineStr">
         <is>
           <t>CAN Bus ; Sagemcom ; SunWhirl (+ H2GP)</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="R12" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:32</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="S12" s="0" t="inlineStr">
         <is>
           <t>CV_EN.pdf</t>
         </is>
@@ -1298,7 +1298,7 @@
         <v>45957.43654626158</v>
       </c>
       <c r="M13" s="29" t="n"/>
-      <c r="O13" t="inlineStr">
+      <c r="O13" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -1346,7 +1346,7 @@
         <v>45957.43655104167</v>
       </c>
       <c r="M14" s="29" t="n"/>
-      <c r="O14" t="inlineStr">
+      <c r="O14" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -1396,27 +1396,27 @@
         <v>45957.43655642361</v>
       </c>
       <c r="M15" s="29" t="n"/>
-      <c r="O15" t="inlineStr">
+      <c r="O15" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="P15" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
+      <c r="Q15" s="0" t="inlineStr">
         <is>
           <t>Micro-réseaux PES/PELS ; MPPT ; SunWhirl</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="R15" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:32</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="S15" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -1454,7 +1454,7 @@
         <v>45957.4365615162</v>
       </c>
       <c r="M16" s="29" t="n"/>
-      <c r="O16" t="inlineStr">
+      <c r="O16" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -1500,27 +1500,27 @@
         <v>45957.4366125926</v>
       </c>
       <c r="M17" s="29" t="n"/>
-      <c r="O17" t="inlineStr">
+      <c r="O17" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="P17" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="Q17" s="0" t="inlineStr">
         <is>
           <t>Sagemcom ; MPPT ; MIGSens</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="R17" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:32</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="S17" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -1566,27 +1566,27 @@
         <v>45957.43661765046</v>
       </c>
       <c r="M18" s="29" t="n"/>
-      <c r="O18" t="inlineStr">
+      <c r="O18" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="P18" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
+      <c r="Q18" s="0" t="inlineStr">
         <is>
           <t>Micro-réseaux PES/PELS ; MIGSens ; SunWhirl (+ H2GP)</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="R18" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:32</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="S18" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -1628,7 +1628,7 @@
         <v>45957.43662319444</v>
       </c>
       <c r="M19" s="29" t="n"/>
-      <c r="O19" t="inlineStr">
+      <c r="O19" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -1674,7 +1674,7 @@
         <v>45957.43662777778</v>
       </c>
       <c r="M20" s="29" t="n"/>
-      <c r="O20" t="inlineStr">
+      <c r="O20" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -1743,7 +1743,7 @@
         <v>45957.43667891204</v>
       </c>
       <c r="M22" s="29" t="n"/>
-      <c r="O22" t="inlineStr">
+      <c r="O22" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -1904,7 +1904,7 @@
         <v>45957.43668399306</v>
       </c>
       <c r="M28" s="29" t="n"/>
-      <c r="O28" t="inlineStr">
+      <c r="O28" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -1946,27 +1946,27 @@
         <v>45957.43668935185</v>
       </c>
       <c r="M29" s="29" t="n"/>
-      <c r="O29" t="inlineStr">
+      <c r="O29" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="P29" s="0" t="inlineStr">
         <is>
           <t>anglais</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr">
+      <c r="Q29" s="0" t="inlineStr">
         <is>
           <t>SunWhirl ; CAN Bus ; STM32N6 (IA embarquée)</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
+      <c r="R29" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:32</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr">
+      <c r="S29" s="0" t="inlineStr">
         <is>
           <t>CV_EN.pdf</t>
         </is>
@@ -2004,7 +2004,7 @@
         <v>45957.43669423611</v>
       </c>
       <c r="M30" s="29" t="n"/>
-      <c r="O30" t="inlineStr">
+      <c r="O30" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -2115,7 +2115,7 @@
         <v>45957.43672258102</v>
       </c>
       <c r="M34" s="29" t="n"/>
-      <c r="O34" t="inlineStr">
+      <c r="O34" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -2157,7 +2157,7 @@
         <v>45957.43672762731</v>
       </c>
       <c r="M35" s="29" t="n"/>
-      <c r="O35" t="inlineStr">
+      <c r="O35" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -2200,27 +2200,27 @@
         <v>45957.4367333449</v>
       </c>
       <c r="M36" s="29" t="n"/>
-      <c r="O36" t="inlineStr">
+      <c r="O36" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
+      <c r="P36" s="0" t="inlineStr">
         <is>
           <t>anglais</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr">
+      <c r="Q36" s="0" t="inlineStr">
         <is>
           <t>CAN Bus ; MIGSens ; CalmaWear</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr">
+      <c r="R36" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:32</t>
         </is>
       </c>
-      <c r="S36" t="inlineStr">
+      <c r="S36" s="0" t="inlineStr">
         <is>
           <t>CV_EN.pdf</t>
         </is>
@@ -2270,7 +2270,7 @@
         <v>45957.43673850694</v>
       </c>
       <c r="M37" s="29" t="n"/>
-      <c r="O37" t="inlineStr">
+      <c r="O37" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -2308,6 +2308,31 @@
         <v>45957.43678990741</v>
       </c>
       <c r="M38" s="29" t="n"/>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>MIGSens ; Sagemcom ; CAN Bus</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:35</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="22.5" customHeight="1" s="32">
       <c r="A39" s="31" t="inlineStr">
@@ -2395,7 +2420,7 @@
         <v>45957.43679489583</v>
       </c>
       <c r="M41" s="29" t="n"/>
-      <c r="O41" t="inlineStr">
+      <c r="O41" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -2433,7 +2458,7 @@
         <v>45957.43679978009</v>
       </c>
       <c r="M42" s="29" t="n"/>
-      <c r="O42" t="inlineStr">
+      <c r="O42" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -2498,7 +2523,7 @@
         <v>45957.43680464121</v>
       </c>
       <c r="M44" s="29" t="n"/>
-      <c r="O44" t="inlineStr">
+      <c r="O44" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -2536,7 +2561,7 @@
         <v>45957.4369069676</v>
       </c>
       <c r="M45" s="29" t="n"/>
-      <c r="O45" t="inlineStr">
+      <c r="O45" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -2574,6 +2599,31 @@
         <v>45957.43692974537</v>
       </c>
       <c r="M46" s="29" t="n"/>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>anglais</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Télésurveillance temps réel ; CalmaWear ; SunWhirl</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:35</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>CV_EN.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="22.5" customHeight="1" s="32">
       <c r="A47" s="31" t="inlineStr">
@@ -2608,6 +2658,31 @@
         <v>45957.43696021991</v>
       </c>
       <c r="M47" s="29" t="n"/>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>CalmaWear ; SunWhirl ; STM32N6 (IA embarquée)</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:35</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="22.5" customHeight="1" s="32">
       <c r="A48" s="31" t="inlineStr">
@@ -2641,6 +2716,31 @@
         <v>45957.43699341435</v>
       </c>
       <c r="M48" s="29" t="n"/>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>anglais</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>CAN Bus ; STM32N6 (IA embarquée) ; CalmaWear</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:35</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>CV_EN.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="22.5" customHeight="1" s="32">
       <c r="A49" s="31" t="inlineStr">
@@ -2794,7 +2894,7 @@
         <v>45957.43706625</v>
       </c>
       <c r="M53" s="29" t="n"/>
-      <c r="O53" t="inlineStr">
+      <c r="O53" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -2832,7 +2932,7 @@
         <v>45957.43711337963</v>
       </c>
       <c r="M54" s="29" t="n"/>
-      <c r="O54" t="inlineStr">
+      <c r="O54" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -2975,6 +3075,31 @@
         <v>45957.43715086806</v>
       </c>
       <c r="M58" s="29" t="n"/>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>anglais</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>CAN Bus ; MIGSens ; SunWhirl</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:35</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>CV_EN.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="22.5" customHeight="1" s="32">
       <c r="A59" s="31" t="inlineStr">
@@ -3016,7 +3141,7 @@
         <v>45957.43719201389</v>
       </c>
       <c r="M59" s="29" t="n"/>
-      <c r="O59" t="inlineStr">
+      <c r="O59" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -3066,6 +3191,31 @@
         <v>45957.43722028935</v>
       </c>
       <c r="M60" s="29" t="n"/>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Télésurveillance temps réel ; MIGSens ; SunWhirl</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:35</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="22.5" customHeight="1" s="32">
       <c r="A61" s="31" t="inlineStr">
@@ -3107,6 +3257,31 @@
         <v>45957.4372678125</v>
       </c>
       <c r="M61" s="29" t="n"/>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>SunWhirl ; CAN Bus ; MIGSens</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:35</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="22.5" customHeight="1" s="32">
       <c r="A62" s="31" t="inlineStr">
@@ -3375,6 +3550,31 @@
         <v>45957.4373644213</v>
       </c>
       <c r="M68" s="29" t="n"/>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>Sagemcom ; Télésurveillance temps réel ; CAN Bus</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:35</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="22.5" customHeight="1" s="32">
       <c r="A69" s="31" t="inlineStr">
@@ -3412,7 +3612,7 @@
         <v>45957.43740361111</v>
       </c>
       <c r="M69" s="29" t="n"/>
-      <c r="O69" t="inlineStr">
+      <c r="O69" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -3454,6 +3654,31 @@
         <v>45957.43742572916</v>
       </c>
       <c r="M70" s="29" t="n"/>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>MIGSens ; CAN Bus ; SunWhirl</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:35</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="22.5" customHeight="1" s="32">
       <c r="A71" s="31" t="inlineStr">
@@ -3560,7 +3785,7 @@
         <v>45988.51455915509</v>
       </c>
       <c r="M74" s="29" t="n"/>
-      <c r="O74" t="inlineStr">
+      <c r="O74" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -3598,7 +3823,7 @@
         <v>45988.51456922454</v>
       </c>
       <c r="M75" s="29" t="n"/>
-      <c r="O75" t="inlineStr">
+      <c r="O75" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -3636,6 +3861,31 @@
         <v>45988.51457988426</v>
       </c>
       <c r="M76" s="29" t="n"/>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>anglais</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>MIGSens ; CAN Bus ; Télésurveillance temps réel</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:35</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>CV_EN.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="22.5" customHeight="1" s="32">
       <c r="A77" s="22" t="inlineStr">
@@ -3776,7 +4026,7 @@
       <c r="L81" s="30" t="n">
         <v>45988.51463702547</v>
       </c>
-      <c r="O81" t="inlineStr">
+      <c r="O81" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -3841,7 +4091,7 @@
       <c r="L83" s="30" t="n">
         <v>45988.51468505787</v>
       </c>
-      <c r="O83" t="inlineStr">
+      <c r="O83" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -3876,7 +4126,7 @@
       <c r="L84" s="30" t="n">
         <v>45988.51470270834</v>
       </c>
-      <c r="O84" t="inlineStr">
+      <c r="O84" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -3911,7 +4161,7 @@
       <c r="L85" s="30" t="n">
         <v>45988.51471092593</v>
       </c>
-      <c r="O85" t="inlineStr">
+      <c r="O85" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>
@@ -4006,7 +4256,7 @@
       <c r="L88" s="30" t="n">
         <v>45995.67262321759</v>
       </c>
-      <c r="O88" t="inlineStr">
+      <c r="O88" s="0" t="inlineStr">
         <is>
           <t>email à vérifier</t>
         </is>

</xml_diff>

<commit_message>
Batch 3: last 6 PFE application drafts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014L6ZvGt8TCo7GsJyTNk89Z
</commit_message>
<xml_diff>
--- a/Copie de stage.xlsx
+++ b/Copie de stage.xlsx
@@ -2308,27 +2308,27 @@
         <v>45957.43678990741</v>
       </c>
       <c r="M38" s="29" t="n"/>
-      <c r="O38" t="inlineStr">
+      <c r="O38" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr">
+      <c r="P38" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q38" t="inlineStr">
+      <c r="Q38" s="0" t="inlineStr">
         <is>
           <t>MIGSens ; Sagemcom ; CAN Bus</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr">
+      <c r="R38" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:35</t>
         </is>
       </c>
-      <c r="S38" t="inlineStr">
+      <c r="S38" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -2599,27 +2599,27 @@
         <v>45957.43692974537</v>
       </c>
       <c r="M46" s="29" t="n"/>
-      <c r="O46" t="inlineStr">
+      <c r="O46" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr">
+      <c r="P46" s="0" t="inlineStr">
         <is>
           <t>anglais</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr">
+      <c r="Q46" s="0" t="inlineStr">
         <is>
           <t>Télésurveillance temps réel ; CalmaWear ; SunWhirl</t>
         </is>
       </c>
-      <c r="R46" t="inlineStr">
+      <c r="R46" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:35</t>
         </is>
       </c>
-      <c r="S46" t="inlineStr">
+      <c r="S46" s="0" t="inlineStr">
         <is>
           <t>CV_EN.pdf</t>
         </is>
@@ -2658,27 +2658,27 @@
         <v>45957.43696021991</v>
       </c>
       <c r="M47" s="29" t="n"/>
-      <c r="O47" t="inlineStr">
+      <c r="O47" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr">
+      <c r="P47" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q47" t="inlineStr">
+      <c r="Q47" s="0" t="inlineStr">
         <is>
           <t>CalmaWear ; SunWhirl ; STM32N6 (IA embarquée)</t>
         </is>
       </c>
-      <c r="R47" t="inlineStr">
+      <c r="R47" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:35</t>
         </is>
       </c>
-      <c r="S47" t="inlineStr">
+      <c r="S47" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -2716,27 +2716,27 @@
         <v>45957.43699341435</v>
       </c>
       <c r="M48" s="29" t="n"/>
-      <c r="O48" t="inlineStr">
+      <c r="O48" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr">
+      <c r="P48" s="0" t="inlineStr">
         <is>
           <t>anglais</t>
         </is>
       </c>
-      <c r="Q48" t="inlineStr">
+      <c r="Q48" s="0" t="inlineStr">
         <is>
           <t>CAN Bus ; STM32N6 (IA embarquée) ; CalmaWear</t>
         </is>
       </c>
-      <c r="R48" t="inlineStr">
+      <c r="R48" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:35</t>
         </is>
       </c>
-      <c r="S48" t="inlineStr">
+      <c r="S48" s="0" t="inlineStr">
         <is>
           <t>CV_EN.pdf</t>
         </is>
@@ -3075,27 +3075,27 @@
         <v>45957.43715086806</v>
       </c>
       <c r="M58" s="29" t="n"/>
-      <c r="O58" t="inlineStr">
+      <c r="O58" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P58" t="inlineStr">
+      <c r="P58" s="0" t="inlineStr">
         <is>
           <t>anglais</t>
         </is>
       </c>
-      <c r="Q58" t="inlineStr">
+      <c r="Q58" s="0" t="inlineStr">
         <is>
           <t>CAN Bus ; MIGSens ; SunWhirl</t>
         </is>
       </c>
-      <c r="R58" t="inlineStr">
+      <c r="R58" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:35</t>
         </is>
       </c>
-      <c r="S58" t="inlineStr">
+      <c r="S58" s="0" t="inlineStr">
         <is>
           <t>CV_EN.pdf</t>
         </is>
@@ -3191,27 +3191,27 @@
         <v>45957.43722028935</v>
       </c>
       <c r="M60" s="29" t="n"/>
-      <c r="O60" t="inlineStr">
+      <c r="O60" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P60" t="inlineStr">
+      <c r="P60" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q60" t="inlineStr">
+      <c r="Q60" s="0" t="inlineStr">
         <is>
           <t>Télésurveillance temps réel ; MIGSens ; SunWhirl</t>
         </is>
       </c>
-      <c r="R60" t="inlineStr">
+      <c r="R60" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:35</t>
         </is>
       </c>
-      <c r="S60" t="inlineStr">
+      <c r="S60" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -3257,27 +3257,27 @@
         <v>45957.4372678125</v>
       </c>
       <c r="M61" s="29" t="n"/>
-      <c r="O61" t="inlineStr">
+      <c r="O61" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P61" t="inlineStr">
+      <c r="P61" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q61" t="inlineStr">
+      <c r="Q61" s="0" t="inlineStr">
         <is>
           <t>SunWhirl ; CAN Bus ; MIGSens</t>
         </is>
       </c>
-      <c r="R61" t="inlineStr">
+      <c r="R61" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:35</t>
         </is>
       </c>
-      <c r="S61" t="inlineStr">
+      <c r="S61" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -3550,27 +3550,27 @@
         <v>45957.4373644213</v>
       </c>
       <c r="M68" s="29" t="n"/>
-      <c r="O68" t="inlineStr">
+      <c r="O68" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P68" t="inlineStr">
+      <c r="P68" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q68" t="inlineStr">
+      <c r="Q68" s="0" t="inlineStr">
         <is>
           <t>Sagemcom ; Télésurveillance temps réel ; CAN Bus</t>
         </is>
       </c>
-      <c r="R68" t="inlineStr">
+      <c r="R68" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:35</t>
         </is>
       </c>
-      <c r="S68" t="inlineStr">
+      <c r="S68" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -3654,27 +3654,27 @@
         <v>45957.43742572916</v>
       </c>
       <c r="M70" s="29" t="n"/>
-      <c r="O70" t="inlineStr">
+      <c r="O70" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P70" t="inlineStr">
+      <c r="P70" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q70" t="inlineStr">
+      <c r="Q70" s="0" t="inlineStr">
         <is>
           <t>MIGSens ; CAN Bus ; SunWhirl</t>
         </is>
       </c>
-      <c r="R70" t="inlineStr">
+      <c r="R70" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:35</t>
         </is>
       </c>
-      <c r="S70" t="inlineStr">
+      <c r="S70" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -3861,27 +3861,27 @@
         <v>45988.51457988426</v>
       </c>
       <c r="M76" s="29" t="n"/>
-      <c r="O76" t="inlineStr">
+      <c r="O76" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P76" t="inlineStr">
+      <c r="P76" s="0" t="inlineStr">
         <is>
           <t>anglais</t>
         </is>
       </c>
-      <c r="Q76" t="inlineStr">
+      <c r="Q76" s="0" t="inlineStr">
         <is>
           <t>MIGSens ; CAN Bus ; Télésurveillance temps réel</t>
         </is>
       </c>
-      <c r="R76" t="inlineStr">
+      <c r="R76" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:35</t>
         </is>
       </c>
-      <c r="S76" t="inlineStr">
+      <c r="S76" s="0" t="inlineStr">
         <is>
           <t>CV_EN.pdf</t>
         </is>
@@ -3919,6 +3919,31 @@
         <v>45988.51458790509</v>
       </c>
       <c r="M77" s="29" t="n"/>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>CAN Bus ; CalmaWear ; SunWhirl</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:37</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="22.5" customHeight="1" s="32">
       <c r="A78" s="22" t="inlineStr">
@@ -3949,6 +3974,31 @@
       <c r="L78" s="30" t="n">
         <v>45988.51462035879</v>
       </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>anglais</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>Sagemcom ; MIGSens ; CAN Bus</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:37</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>CV_EN.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="22.5" customHeight="1" s="32">
       <c r="A79" s="31" t="inlineStr">
@@ -3979,6 +4029,31 @@
       <c r="L79" s="30" t="n">
         <v>45988.51462847222</v>
       </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>anglais</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>CAN Bus ; SunWhirl ; MIGSens (+ H2GP)</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:37</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>CV_EN.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="22.5" customHeight="1" s="32">
       <c r="A80" s="31" t="inlineStr">
@@ -4061,6 +4136,31 @@
       <c r="L82" s="30" t="n">
         <v>45988.5146452662</v>
       </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>SunWhirl ; CAN Bus ; MIGSens (+ H2GP)</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:37</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="22.5" customHeight="1" s="32">
       <c r="A83" s="31" t="inlineStr">
@@ -4196,6 +4296,31 @@
       <c r="L86" s="30" t="n">
         <v>45988.51472016203</v>
       </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>français</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>SunWhirl ; MIGSens ; CalmaWear</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:37</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>Cv_Farah_Fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="22.5" customHeight="1" s="32">
       <c r="A87" s="31" t="inlineStr">
@@ -4225,6 +4350,31 @@
       </c>
       <c r="L87" s="30" t="n">
         <v>45988.51472819444</v>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>brouillon créé</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>anglais</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>SunWhirl ; Sagemcom ; CAN Bus</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>2026-09-28 14:37</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>CV_EN.pdf</t>
+        </is>
       </c>
     </row>
     <row r="88" ht="22.5" customHeight="1" s="32">

</xml_diff>

<commit_message>
Add line-following robot project to 9 robotics/automation drafts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014L6ZvGt8TCo7GsJyTNk89Z
</commit_message>
<xml_diff>
--- a/Copie de stage.xlsx
+++ b/Copie de stage.xlsx
@@ -926,7 +926,7 @@
       <c r="M6" s="29" t="n"/>
       <c r="O6" s="0" t="inlineStr">
         <is>
-          <t>brouillon créé</t>
+          <t>envoi programmé par toi (non modifié)</t>
         </is>
       </c>
       <c r="P6" s="0" t="inlineStr">
@@ -1019,7 +1019,7 @@
       <c r="M8" s="29" t="n"/>
       <c r="O8" s="0" t="inlineStr">
         <is>
-          <t>brouillon créé</t>
+          <t>envoi programmé par toi (non modifié)</t>
         </is>
       </c>
       <c r="P8" s="0" t="inlineStr">
@@ -1948,7 +1948,7 @@
       <c r="M29" s="29" t="n"/>
       <c r="O29" s="0" t="inlineStr">
         <is>
-          <t>brouillon créé</t>
+          <t>envoyé par toi (non modifié)</t>
         </is>
       </c>
       <c r="P29" s="0" t="inlineStr">
@@ -2310,7 +2310,7 @@
       <c r="M38" s="29" t="n"/>
       <c r="O38" s="0" t="inlineStr">
         <is>
-          <t>brouillon créé</t>
+          <t>envoi programmé par toi (non modifié)</t>
         </is>
       </c>
       <c r="P38" s="0" t="inlineStr">
@@ -2601,7 +2601,7 @@
       <c r="M46" s="29" t="n"/>
       <c r="O46" s="0" t="inlineStr">
         <is>
-          <t>brouillon créé</t>
+          <t>envoi programmé par toi (non modifié)</t>
         </is>
       </c>
       <c r="P46" s="0" t="inlineStr">
@@ -2660,7 +2660,7 @@
       <c r="M47" s="29" t="n"/>
       <c r="O47" s="0" t="inlineStr">
         <is>
-          <t>brouillon créé</t>
+          <t>brouillon mis à jour (robot suiveur)</t>
         </is>
       </c>
       <c r="P47" s="0" t="inlineStr">
@@ -2670,12 +2670,12 @@
       </c>
       <c r="Q47" s="0" t="inlineStr">
         <is>
-          <t>CalmaWear ; SunWhirl ; STM32N6 (IA embarquée)</t>
+          <t>CalmaWear ; SunWhirl ; Robot suiveur de ligne (PID)</t>
         </is>
       </c>
       <c r="R47" s="0" t="inlineStr">
         <is>
-          <t>2026-09-28 14:35</t>
+          <t>2026-09-28 16:31</t>
         </is>
       </c>
       <c r="S47" s="0" t="inlineStr">
@@ -3193,7 +3193,7 @@
       <c r="M60" s="29" t="n"/>
       <c r="O60" s="0" t="inlineStr">
         <is>
-          <t>brouillon créé</t>
+          <t>brouillon mis à jour (robot suiveur)</t>
         </is>
       </c>
       <c r="P60" s="0" t="inlineStr">
@@ -3203,12 +3203,12 @@
       </c>
       <c r="Q60" s="0" t="inlineStr">
         <is>
-          <t>Télésurveillance temps réel ; MIGSens ; SunWhirl</t>
+          <t>Télésurveillance temps réel ; MIGSens ; Robot suiveur de ligne (PID)</t>
         </is>
       </c>
       <c r="R60" s="0" t="inlineStr">
         <is>
-          <t>2026-09-28 14:35</t>
+          <t>2026-09-28 16:31</t>
         </is>
       </c>
       <c r="S60" s="0" t="inlineStr">
@@ -3259,7 +3259,7 @@
       <c r="M61" s="29" t="n"/>
       <c r="O61" s="0" t="inlineStr">
         <is>
-          <t>brouillon créé</t>
+          <t>brouillon mis à jour (robot suiveur)</t>
         </is>
       </c>
       <c r="P61" s="0" t="inlineStr">
@@ -3269,12 +3269,12 @@
       </c>
       <c r="Q61" s="0" t="inlineStr">
         <is>
-          <t>SunWhirl ; CAN Bus ; MIGSens</t>
+          <t>SunWhirl ; Robot suiveur de ligne (PID) ; MIGSens</t>
         </is>
       </c>
       <c r="R61" s="0" t="inlineStr">
         <is>
-          <t>2026-09-28 14:35</t>
+          <t>2026-09-28 16:31</t>
         </is>
       </c>
       <c r="S61" s="0" t="inlineStr">
@@ -3656,7 +3656,7 @@
       <c r="M70" s="29" t="n"/>
       <c r="O70" s="0" t="inlineStr">
         <is>
-          <t>brouillon créé</t>
+          <t>brouillon mis à jour (robot suiveur)</t>
         </is>
       </c>
       <c r="P70" s="0" t="inlineStr">
@@ -3666,12 +3666,12 @@
       </c>
       <c r="Q70" s="0" t="inlineStr">
         <is>
-          <t>MIGSens ; CAN Bus ; SunWhirl</t>
+          <t>MIGSens ; Robot suiveur de ligne (PID) ; SunWhirl</t>
         </is>
       </c>
       <c r="R70" s="0" t="inlineStr">
         <is>
-          <t>2026-09-28 14:35</t>
+          <t>2026-09-28 16:31</t>
         </is>
       </c>
       <c r="S70" s="0" t="inlineStr">
@@ -3863,7 +3863,7 @@
       <c r="M76" s="29" t="n"/>
       <c r="O76" s="0" t="inlineStr">
         <is>
-          <t>brouillon créé</t>
+          <t>brouillon mis à jour (robot suiveur)</t>
         </is>
       </c>
       <c r="P76" s="0" t="inlineStr">
@@ -3873,12 +3873,12 @@
       </c>
       <c r="Q76" s="0" t="inlineStr">
         <is>
-          <t>MIGSens ; CAN Bus ; Télésurveillance temps réel</t>
+          <t>MIGSens ; CAN Bus ; Robot suiveur de ligne (PID)</t>
         </is>
       </c>
       <c r="R76" s="0" t="inlineStr">
         <is>
-          <t>2026-09-28 14:35</t>
+          <t>2026-09-28 16:31</t>
         </is>
       </c>
       <c r="S76" s="0" t="inlineStr">
@@ -3919,27 +3919,27 @@
         <v>45988.51458790509</v>
       </c>
       <c r="M77" s="29" t="n"/>
-      <c r="O77" t="inlineStr">
+      <c r="O77" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P77" t="inlineStr">
+      <c r="P77" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q77" t="inlineStr">
+      <c r="Q77" s="0" t="inlineStr">
         <is>
           <t>CAN Bus ; CalmaWear ; SunWhirl</t>
         </is>
       </c>
-      <c r="R77" t="inlineStr">
+      <c r="R77" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:37</t>
         </is>
       </c>
-      <c r="S77" t="inlineStr">
+      <c r="S77" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -3974,27 +3974,27 @@
       <c r="L78" s="30" t="n">
         <v>45988.51462035879</v>
       </c>
-      <c r="O78" t="inlineStr">
-        <is>
-          <t>brouillon créé</t>
-        </is>
-      </c>
-      <c r="P78" t="inlineStr">
+      <c r="O78" s="0" t="inlineStr">
+        <is>
+          <t>brouillon mis à jour (robot suiveur)</t>
+        </is>
+      </c>
+      <c r="P78" s="0" t="inlineStr">
         <is>
           <t>anglais</t>
         </is>
       </c>
-      <c r="Q78" t="inlineStr">
-        <is>
-          <t>Sagemcom ; MIGSens ; CAN Bus</t>
-        </is>
-      </c>
-      <c r="R78" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:37</t>
-        </is>
-      </c>
-      <c r="S78" t="inlineStr">
+      <c r="Q78" s="0" t="inlineStr">
+        <is>
+          <t>Sagemcom ; MIGSens ; Robot suiveur de ligne (PID)</t>
+        </is>
+      </c>
+      <c r="R78" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-28 16:31</t>
+        </is>
+      </c>
+      <c r="S78" s="0" t="inlineStr">
         <is>
           <t>CV_EN.pdf</t>
         </is>
@@ -4029,27 +4029,27 @@
       <c r="L79" s="30" t="n">
         <v>45988.51462847222</v>
       </c>
-      <c r="O79" t="inlineStr">
+      <c r="O79" s="0" t="inlineStr">
         <is>
           <t>brouillon créé</t>
         </is>
       </c>
-      <c r="P79" t="inlineStr">
+      <c r="P79" s="0" t="inlineStr">
         <is>
           <t>anglais</t>
         </is>
       </c>
-      <c r="Q79" t="inlineStr">
+      <c r="Q79" s="0" t="inlineStr">
         <is>
           <t>CAN Bus ; SunWhirl ; MIGSens (+ H2GP)</t>
         </is>
       </c>
-      <c r="R79" t="inlineStr">
+      <c r="R79" s="0" t="inlineStr">
         <is>
           <t>2026-09-28 14:37</t>
         </is>
       </c>
-      <c r="S79" t="inlineStr">
+      <c r="S79" s="0" t="inlineStr">
         <is>
           <t>CV_EN.pdf</t>
         </is>
@@ -4136,27 +4136,27 @@
       <c r="L82" s="30" t="n">
         <v>45988.5146452662</v>
       </c>
-      <c r="O82" t="inlineStr">
-        <is>
-          <t>brouillon créé</t>
-        </is>
-      </c>
-      <c r="P82" t="inlineStr">
+      <c r="O82" s="0" t="inlineStr">
+        <is>
+          <t>brouillon mis à jour (robot suiveur)</t>
+        </is>
+      </c>
+      <c r="P82" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q82" t="inlineStr">
-        <is>
-          <t>SunWhirl ; CAN Bus ; MIGSens (+ H2GP)</t>
-        </is>
-      </c>
-      <c r="R82" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:37</t>
-        </is>
-      </c>
-      <c r="S82" t="inlineStr">
+      <c r="Q82" s="0" t="inlineStr">
+        <is>
+          <t>SunWhirl ; CAN Bus ; Robot suiveur de ligne (PID)</t>
+        </is>
+      </c>
+      <c r="R82" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-28 16:31</t>
+        </is>
+      </c>
+      <c r="S82" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -4296,27 +4296,27 @@
       <c r="L86" s="30" t="n">
         <v>45988.51472016203</v>
       </c>
-      <c r="O86" t="inlineStr">
-        <is>
-          <t>brouillon créé</t>
-        </is>
-      </c>
-      <c r="P86" t="inlineStr">
+      <c r="O86" s="0" t="inlineStr">
+        <is>
+          <t>brouillon mis à jour (robot suiveur)</t>
+        </is>
+      </c>
+      <c r="P86" s="0" t="inlineStr">
         <is>
           <t>français</t>
         </is>
       </c>
-      <c r="Q86" t="inlineStr">
-        <is>
-          <t>SunWhirl ; MIGSens ; CalmaWear</t>
-        </is>
-      </c>
-      <c r="R86" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:37</t>
-        </is>
-      </c>
-      <c r="S86" t="inlineStr">
+      <c r="Q86" s="0" t="inlineStr">
+        <is>
+          <t>SunWhirl ; MIGSens ; Robot suiveur de ligne (PID)</t>
+        </is>
+      </c>
+      <c r="R86" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-28 16:31</t>
+        </is>
+      </c>
+      <c r="S86" s="0" t="inlineStr">
         <is>
           <t>Cv_Farah_Fr.pdf</t>
         </is>
@@ -4351,27 +4351,27 @@
       <c r="L87" s="30" t="n">
         <v>45988.51472819444</v>
       </c>
-      <c r="O87" t="inlineStr">
-        <is>
-          <t>brouillon créé</t>
-        </is>
-      </c>
-      <c r="P87" t="inlineStr">
+      <c r="O87" s="0" t="inlineStr">
+        <is>
+          <t>brouillon mis à jour (robot suiveur)</t>
+        </is>
+      </c>
+      <c r="P87" s="0" t="inlineStr">
         <is>
           <t>anglais</t>
         </is>
       </c>
-      <c r="Q87" t="inlineStr">
-        <is>
-          <t>SunWhirl ; Sagemcom ; CAN Bus</t>
-        </is>
-      </c>
-      <c r="R87" t="inlineStr">
-        <is>
-          <t>2026-09-28 14:37</t>
-        </is>
-      </c>
-      <c r="S87" t="inlineStr">
+      <c r="Q87" s="0" t="inlineStr">
+        <is>
+          <t>SunWhirl ; Sagemcom ; Robot suiveur de ligne (PID)</t>
+        </is>
+      </c>
+      <c r="R87" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-28 16:31</t>
+        </is>
+      </c>
+      <c r="S87" s="0" t="inlineStr">
         <is>
           <t>CV_EN.pdf</t>
         </is>

</xml_diff>